<commit_message>
Refractored and made resolution template more configurable
</commit_message>
<xml_diff>
--- a/db_storage/resolution_template.xlsx
+++ b/db_storage/resolution_template.xlsx
@@ -9,6 +9,7 @@
     <sheet name="variables" sheetId="4" r:id="rId4"/>
     <sheet name="games" sheetId="5" r:id="rId5"/>
     <sheet name="sub_category" sheetId="6" r:id="rId6"/>
+    <sheet name="categories" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -424,7 +425,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -466,16 +467,24 @@
         <v>id,title,games,created_at,updated_at</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>categories</v>
+      </c>
+      <c r="B6" t="str">
+        <v>id,title,created_at,updated_at</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -520,13 +529,13 @@
         <v>General Round Check</v>
       </c>
       <c r="F2" t="str">
-        <v>{"root":{"children":[{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Issue:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Steps to Reproduce:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoid","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoName","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"roundId","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Player ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"playerId","display":"{player_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"gameId","display":"{game_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Live","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":16,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Internal Investigation:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Upon investigation, we have found that:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Next Action:","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Communicating with the operator","type":"text","version":1},{"detail":0,"format":16,"mode":"normal","style":"","text":".","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Issue:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Steps to Reproduce:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoid","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoName","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"roundId","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Player ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"playerId","display":"{player_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"gameId","display":"{game_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Live","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Internal Investigation:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Upon investigation, we have found that:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round url","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"current_url","display":"{current_url}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"BET Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"c_bet_details","display":"{bet_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Transaction Details:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"c_transaction_details","display":"{transaction_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Next Action:","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Communicating with the operator","type":"text","version":1},{"detail":0,"format":16,"mode":"normal","style":"","text":".","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
       </c>
       <c r="G2" t="str">
         <v>2026-04-04T15:50:25.541Z</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-04-06T05:35:29.650Z</v>
+        <v>2026-04-07T02:14:23.372Z</v>
       </c>
     </row>
     <row r="3">
@@ -546,13 +555,13 @@
         <v>BET Canceled</v>
       </c>
       <c r="F3" t="str">
-        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Dear Team, ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Thank you for reaching out to us regarding Ticket: ","type":"text","version":1},{"type":"field","version":1,"keyName":"ticketId","display":"{TikcetID}"},{"type":"linebreak","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Issue Description","type":"text","version":1},{"detail":0,"format":1,"mode":"normal","style":"","text":": ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Bet Canceled ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Resolution Summary","type":"text","version":1},{"detail":0,"format":1,"mode":"normal","style":"","text":": ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We have reviewed your request for Round -","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"roundId","display":"{roundId}"}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Found that - ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"When we sent the BET request for this round to your system, we didn’t receive a response in time. By the time the game started, the betting window had already closed, so the bet was automatically cancelled. ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We will now resolve this ticket. Please let us know if you are still having this issue. ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thanks, ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Pragmatic Play Support.","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Dear Team, ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Thank you for reaching out to us regarding Ticket: ","type":"text","version":1},{"type":"field","version":1,"keyName":"ticketId","display":"{tikcet_id}"},{"type":"linebreak","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Issue Description","type":"text","version":1},{"detail":0,"format":1,"mode":"normal","style":"","text":": ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Bet Canceled ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Resolution Summary","type":"text","version":1},{"detail":0,"format":1,"mode":"normal","style":"","text":": ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We have reviewed your request for Round -","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"roundId","display":"{round_id}"}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Found that - ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"When we sent the BET request for this round to your system, we didn’t receive a response in time. By the time the game started, the betting window had already closed, so the bet was automatically cancelled. ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We will now resolve this ticket. Please let us know if you are still having this issue. ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thanks, ","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Pragmatic Play Support.","type":"text","version":1}],"direction":null,"format":"left","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
       </c>
       <c r="G3" t="str">
         <v>2026-04-04T23:43:51.100Z</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-04-05T15:51:53.081Z</v>
+        <v>2026-04-06T12:57:59.972Z</v>
       </c>
     </row>
     <row r="4">
@@ -578,19 +587,97 @@
         <v>2026-04-04T23:45:47.309Z</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-04-06T05:37:11.063Z</v>
+        <v>2026-04-06T12:57:41.741Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Enable Table</v>
+      </c>
+      <c r="C5" t="str">
+        <v>All</v>
+      </c>
+      <c r="D5" t="str">
+        <v>AM Request</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Enable Table</v>
+      </c>
+      <c r="F5" t="str">
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Hi ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Ticket: ","type":"text","version":1},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"https://pragmaticplay.freshdesk.com/a/tickets/","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"link","version":1,"rel":"noreferrer noopener","target":"_blank","title":"https://pragmaticplay.freshdesk.com/a/tickets/2031563","url":"https://pragmaticplay.freshdesk.com/a/tickets/2031563"},{"type":"linebreak","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"One of your operators is trying to get the following games, which are not enabled on RNG and LC","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"type":"linebreak","version":1},{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino and Game Details : ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Kindly review and confirm approval to enable this parameter for the mentioned brand. Once approved, we will proceed with the enabling. ","type":"text","version":1},{"type":"linebreak","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Thanks and regards, ","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Tech Support ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-04-07T03:33:28.771Z</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-04-07T03:36:55.218Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Enable Table</v>
+      </c>
+      <c r="C6" t="str">
+        <v>All</v>
+      </c>
+      <c r="D6" t="str">
+        <v>LC Integration</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Enable Table</v>
+      </c>
+      <c r="F6" t="str">
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Hello Team,​","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Action: ","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Enabling Tables","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"I would like to request your assistance in enabling the list of game tables provided.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game Table Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"AM Approval","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Please let me know if any additional information is needed to proceed with this request.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thanks,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Technical Support Engineer.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-04-07T03:39:33.046Z</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-04-07T03:39:33.046Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Request : BET Logs</v>
+      </c>
+      <c r="C7" t="str">
+        <v>All</v>
+      </c>
+      <c r="D7" t="str">
+        <v>RNG</v>
+      </c>
+      <c r="E7" t="str">
+        <v>BET Logs Request</v>
+      </c>
+      <c r="F7" t="str">
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Dear Team,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Request:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Please provide the BET/BET_RESULT/END_RESULT/REFUND logs for the following details.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"roundId","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"DateTime","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_session_date_time","display":"{round_session}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Casino Env :  ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_env","display":"{casino_env}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Casino Id : ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoid","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Casino Name: ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoName","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We are currently unable to retrieve the logs from Kibana on our end.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Your assistance in providing these logs at the earliest would be greatly appreciated.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thank you for your support.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Best Regards,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Technical Support Engineer.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-04-07T03:40:50.147Z</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2026-04-07T04:09:08.257Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -711,9 +798,94 @@
         <v>2026-04-06T05:34:41.981Z</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>c_bet_details</v>
+      </c>
+      <c r="C8" t="str">
+        <v>{bet_details}</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-04-07T01:54:22.905Z</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-04-07T01:54:44.075Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>c_transaction_details</v>
+      </c>
+      <c r="C9" t="str">
+        <v>{transaction_details}</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2026-04-07T01:55:10.507Z</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-04-07T01:55:10.507Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>current_url</v>
+      </c>
+      <c r="C10" t="str">
+        <v>{current_url}</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2026-04-07T01:56:41.026Z</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2026-04-07T01:56:41.026Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>casino_env</v>
+      </c>
+      <c r="C11" t="str">
+        <v>{casino_env}</v>
+      </c>
+      <c r="D11" t="str">
+        <v>2026-04-07T03:43:07.390Z</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2026-04-07T03:43:07.390Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>round_session_date_time</v>
+      </c>
+      <c r="C12" t="str">
+        <v>{round_session}</v>
+      </c>
+      <c r="D12" t="str">
+        <v>2026-04-07T03:43:36.650Z</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-04-07T03:43:36.650Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -815,7 +987,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -885,9 +1057,138 @@
         <v>2026-04-05T13:43:34.682Z</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Enable Table</v>
+      </c>
+      <c r="C5" t="str">
+        <v>All</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-04-07T03:28:34.968Z</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-04-07T03:28:34.968Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>BET Logs Request</v>
+      </c>
+      <c r="C6" t="str">
+        <v>All</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-04-07T03:41:20.219Z</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-04-07T03:41:20.219Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>title</v>
+      </c>
+      <c r="C1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="D1" t="str">
+        <v>updated_at</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Resolution Summary</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-04-06T13:16:07.715Z</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-04-06T13:16:07.715Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Operator Response</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2026-04-06T13:16:16.363Z</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-04-06T13:16:16.363Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>AM Request</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-04-07T03:27:39.862Z</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-04-07T03:27:39.862Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>LC Integration</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2026-04-07T03:37:54.605Z</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-04-07T03:37:54.605Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>RNG</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2026-04-07T03:38:01.330Z</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-04-07T03:38:01.330Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated partial-feature filling the values
</commit_message>
<xml_diff>
--- a/db_storage/resolution_template.xlsx
+++ b/db_storage/resolution_template.xlsx
@@ -476,6 +476,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
@@ -529,13 +530,13 @@
         <v>General Round Check</v>
       </c>
       <c r="F2" t="str">
-        <v>{"root":{"children":[{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Issue:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Steps to Reproduce:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoid","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoName","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"roundId","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Player ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"playerId","display":"{player_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"gameId","display":"{game_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Live","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Internal Investigation:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Upon investigation, we have found that:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round url","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"current_url","display":"{current_url}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"BET Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"c_bet_details","display":"{bet_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Transaction Details:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"c_transaction_details","display":"{transaction_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Next Action:","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Communicating with the operator","type":"text","version":1},{"detail":0,"format":16,"mode":"normal","style":"","text":".","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Issue:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Steps to Reproduce:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoid","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoName","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"roundId","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Player ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"playerId","display":"{player_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"gameId","display":"{game_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Live","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Internal Investigation:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Upon investigation, we have found that:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round url","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"currentUrl","display":"{current_url}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"BET Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"c_bet_details","display":"{bet_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Transaction Details:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"c_transaction_details","display":"{transaction_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Next Action:","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Communicating with the operator","type":"text","version":1},{"detail":0,"format":16,"mode":"normal","style":"","text":".","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
       </c>
       <c r="G2" t="str">
         <v>2026-04-04T15:50:25.541Z</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-04-07T02:14:23.372Z</v>
+        <v>2026-04-08T04:39:44.409Z</v>
       </c>
     </row>
     <row r="3">
@@ -633,13 +634,13 @@
         <v>Enable Table</v>
       </c>
       <c r="F6" t="str">
-        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Hello Team,​","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Action: ","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Enabling Tables","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"I would like to request your assistance in enabling the list of game tables provided.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game Table Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"AM Approval","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Please let me know if any additional information is needed to proceed with this request.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thanks,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Technical Support Engineer.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Hello Team,​","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Action: ","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Enabling Tables","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"I would like to request your assistance in enabling the list of game tables provided.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino and Game Table Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"children":[{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Id","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game Id","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Table Name","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Enabled At LC","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Enabled At Platform","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1}],"direction":null,"format":"","indent":0,"type":"tablerow","version":1,"height":21},{"children":[{"children":[{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1}],"direction":null,"format":"","indent":0,"type":"tablerow","version":1,"height":21}],"direction":null,"format":"","indent":0,"type":"table","version":1,"colWidths":[154,154,89,259,100,131]},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"AM Approval","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Please let me know if any additional information is needed to proceed with this request.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thanks,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Technical Support Engineer.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
       </c>
       <c r="G6" t="str">
         <v>2026-04-07T03:39:33.046Z</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-04-07T03:39:33.046Z</v>
+        <v>2026-04-07T09:43:53.299Z</v>
       </c>
     </row>
     <row r="7">
@@ -659,13 +660,13 @@
         <v>BET Logs Request</v>
       </c>
       <c r="F7" t="str">
-        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Dear Team,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Request:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Please provide the BET/BET_RESULT/END_RESULT/REFUND logs for the following details.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"roundId","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"DateTime","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_session_date_time","display":"{round_session}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Casino Env :  ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_env","display":"{casino_env}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Casino Id : ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoid","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Casino Name: ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoName","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We are currently unable to retrieve the logs from Kibana on our end.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Your assistance in providing these logs at the earliest would be greatly appreciated.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thank you for your support.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Best Regards,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Technical Support Engineer.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Dear Team,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Request:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Please provide the BET/BET_RESULT/END_RESULT/REFUND logs for the following details.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"roundId","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"DateTime","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_session_date_time","display":"{round_session}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Casino Env:  ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_env","display":"{casino_env}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Casino ID: ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoid","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Casino Name: ","type":"text","version":1},{"type":"field","version":1,"keyName":"casinoName","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We are currently unable to retrieve the logs from Kibana on our end.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Your assistance in providing these logs at the earliest would be greatly appreciated.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thank you for your support.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Best Regards,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Technical Support Engineer.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
       </c>
       <c r="G7" t="str">
         <v>2026-04-07T03:40:50.147Z</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-04-07T04:09:08.257Z</v>
+        <v>2026-04-07T09:45:06.559Z</v>
       </c>
     </row>
   </sheetData>
@@ -837,7 +838,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>current_url</v>
+        <v>currentUrl</v>
       </c>
       <c r="C10" t="str">
         <v>{current_url}</v>
@@ -846,7 +847,7 @@
         <v>2026-04-07T01:56:41.026Z</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-04-07T01:56:41.026Z</v>
+        <v>2026-04-08T04:37:42.685Z</v>
       </c>
     </row>
     <row r="11">
@@ -854,7 +855,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>casino_env</v>
+        <v>casinoEnv</v>
       </c>
       <c r="C11" t="str">
         <v>{casino_env}</v>
@@ -863,7 +864,7 @@
         <v>2026-04-07T03:43:07.390Z</v>
       </c>
       <c r="E11" t="str">
-        <v>2026-04-07T03:43:07.390Z</v>
+        <v>2026-04-08T04:37:51.950Z</v>
       </c>
     </row>
     <row r="12">
@@ -871,7 +872,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>round_session_date_time</v>
+        <v>roundSessionDateTime</v>
       </c>
       <c r="C12" t="str">
         <v>{round_session}</v>
@@ -880,7 +881,7 @@
         <v>2026-04-07T03:43:36.650Z</v>
       </c>
       <c r="E12" t="str">
-        <v>2026-04-07T03:43:36.650Z</v>
+        <v>2026-04-08T04:38:11.198Z</v>
       </c>
     </row>
   </sheetData>
@@ -979,6 +980,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
@@ -1092,6 +1094,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
@@ -1187,6 +1190,7 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
feat: Implement Baccarat and Blackjack game result components
- Added Baccarat hand report rules and component for displaying game results.
- Introduced Blackjack hand report component with detailed player and dealer sections.
- Created utility functions for calculating scores and determining winners in both Baccarat and Blackjack.
- Refactored card fetching logic to use a unified hook for both games.
- Updated round audit components to integrate new game result displays.
- Removed deprecated additional details wrapper and adjusted related imports.
- Enhanced date formatting utilities for better readability.

Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/db_storage/resolution_template.xlsx
+++ b/db_storage/resolution_template.xlsx
@@ -668,7 +668,7 @@
         <v>BET Logs Request</v>
       </c>
       <c r="F7" t="str">
-        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Dear Team,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Request:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Please provide the BET/BET_RESULT/END_RESULT/REFUND logs for the following details.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_id","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"DateTime","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"  ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID: ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_id","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_desc","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We are currently unable to retrieve the logs from Kibana on our end.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Your assistance in providing these logs at the earliest would be greatly appreciated.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thank you for your support.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Best Regards,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Technical Support Engineer.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Dear Team,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Request:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Please provide the BET/BET_RESULT/END_RESULT/REFUND logs for the following details.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_id","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"DateTime","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"result_time","display":"{round_session}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"  ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID: ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_id","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_desc","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We are currently unable to retrieve the logs from Kibana on our end.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Your assistance in providing these logs at the earliest would be greatly appreciated.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thank you for your support.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Best Regards,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Technical Support Engineer.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
       </c>
       <c r="G7" t="str">
         <v>true</v>
@@ -677,7 +677,7 @@
         <v>2026-04-07T03:40:50.147Z</v>
       </c>
       <c r="J7" t="str">
-        <v>2026-04-12T13:25:21.890Z</v>
+        <v>2026-05-12T05:01:32.467Z</v>
       </c>
     </row>
   </sheetData>
@@ -913,7 +913,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>roundSessionDateTime</v>
+        <v>result_time</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
       </c>
       <c r="E12" t="str">
         <v>{round_session}</v>
@@ -922,7 +928,7 @@
         <v>2026-04-07T03:43:36.650Z</v>
       </c>
       <c r="G12" t="str">
-        <v>2026-04-08T04:38:11.198Z</v>
+        <v>2026-05-12T05:00:51.180Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated ravi - sai
</commit_message>
<xml_diff>
--- a/db_storage/resolution_template.xlsx
+++ b/db_storage/resolution_template.xlsx
@@ -535,13 +535,13 @@
         <v>General Round Check</v>
       </c>
       <c r="F2" t="str">
-        <v>{"root":{"children":[{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Issue:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Steps to Reproduce:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_id","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_desc","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_id","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Player ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"user_id","display":"{user_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"game_id","display":"{game_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Live","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Internal Investigation:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Upon investigation, we have found that:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"BET Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"bet_details","display":"{bet_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Transaction Details:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"transaction_details","display":"{transaction_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Next Action:","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Communicating with the operator","type":"text","version":1},{"detail":0,"format":16,"mode":"normal","style":"","text":".","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Issue:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Steps to Reproduce:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_id","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_name","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_id","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Player ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"user_id","display":"{user_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"game_id","display":"{game_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Live","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Internal Investigation:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Upon investigation, we have found that:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"BET Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"bet_details","display":"{bet_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Transaction Details:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"transaction_details","display":"{transaction_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Next Action:","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Communicating with the operator","type":"text","version":1},{"detail":0,"format":16,"mode":"normal","style":"","text":".","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
       </c>
       <c r="I2" t="str">
         <v>2026-04-04T15:50:25.541Z</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-04-13T16:17:47.432Z</v>
+        <v>2026-05-12T12:15:18.799Z</v>
       </c>
     </row>
     <row r="3">
@@ -613,13 +613,13 @@
         <v>Enable Table</v>
       </c>
       <c r="F5" t="str">
-        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Hi ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Ticket: ","type":"text","version":1},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"https://pragmaticplay.freshdesk.com/a/tickets/2051557","type":"text","version":1},{"type":"linebreak","version":1}],"direction":null,"format":"","indent":0,"type":"link","version":1,"rel":"noreferrer","target":null,"title":null,"url":"https://pragmaticplay.freshdesk.com/a/tickets/2051557"},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"One of your operators is trying to launch the following games, which are not enabled on RNG and LC","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"type":"linebreak","version":1},{"detail":0,"format":9,"mode":"normal","style":"","text":"Casino and Game Details : ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ppcwc00000004725","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" PP Alea luckyshares","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Games :","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"children":[{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Id","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":"rgb(217, 217, 217)","colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game Id","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":"rgb(217, 217, 217)","colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Table Name","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":"rgb(217, 217, 217)","colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Enabled At LC","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":"rgb(217, 217, 217)","colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Enabled At Platform","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":"rgb(217, 217, 217)","colSpan":1,"headerState":0,"rowSpan":1}],"direction":null,"format":"","indent":0,"type":"tablerow","version":1,"height":21},{"children":[{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"ppcwc00000004725","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"2201","type":"text","version":1}],"direction":null,"format":"right","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"High Flyer","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"No","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"No","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1}],"direction":null,"format":"","indent":0,"type":"tablerow","version":1,"height":21}],"direction":null,"format":"","indent":0,"type":"table","version":1,"colWidths":[154,89,259,100,131]},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Kindly review and confirm approval to enable this parameter for the mentioned brand. Once approved, we will proceed with the enabling. ","type":"text","version":1},{"type":"linebreak","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Thanks and regards, ","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Tech Support ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Hi ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Ticket: ","type":"text","version":1},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"https://pragmaticplay.freshdesk.com/a/tickets/","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"link","version":1,"rel":"noreferrer","target":null,"title":null,"url":"https://pragmaticplay.freshdesk.com/a/tickets/2051557"},{"type":"field","version":1,"keyName":"ticketId","display":"{tikcet_id}"},{"children":[{"type":"linebreak","version":1}],"direction":null,"format":"","indent":0,"type":"link","version":1,"rel":"noreferrer","target":null,"title":null,"url":"https://pragmaticplay.freshdesk.com/a/tickets/2051557"},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"One of your operators is trying to launch the following games, which are not enabled on RNG and LC","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"type":"linebreak","version":1},{"detail":0,"format":9,"mode":"normal","style":"","text":"Casino and Game Details : ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ppcwc00000004725","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" PP Alea luckyshares","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Games :","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"children":[{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Id","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":"rgb(217, 217, 217)","colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game Id","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":"rgb(217, 217, 217)","colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Table Name","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":"rgb(217, 217, 217)","colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Enabled At LC","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":"rgb(217, 217, 217)","colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Enabled At Platform","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":"rgb(217, 217, 217)","colSpan":1,"headerState":0,"rowSpan":1}],"direction":null,"format":"","indent":0,"type":"tablerow","version":1,"height":21},{"children":[{"children":[{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[],"direction":null,"format":"right","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1},{"children":[{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"tablecell","version":1,"verticalAlign":"bottom","backgroundColor":null,"colSpan":1,"headerState":0,"rowSpan":1}],"direction":null,"format":"","indent":0,"type":"tablerow","version":1,"height":21}],"direction":null,"format":"","indent":0,"type":"table","version":1,"colWidths":[154,89,259,100,131]},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Kindly review and confirm approval to enable this parameter for the mentioned brand. Once approved, we will proceed with the enabling. ","type":"text","version":1},{"type":"linebreak","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Thanks and regards, ","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Tech Support ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
       </c>
       <c r="I5" t="str">
         <v>2026-04-07T03:33:28.771Z</v>
       </c>
       <c r="J5" t="str">
-        <v>2026-04-14T01:39:45.237Z</v>
+        <v>2026-05-12T12:15:48.697Z</v>
       </c>
     </row>
     <row r="6">
@@ -668,7 +668,7 @@
         <v>BET Logs Request</v>
       </c>
       <c r="F7" t="str">
-        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Dear Team,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Request:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Please provide the BET/BET_RESULT/END_RESULT/REFUND logs for the following details.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_id","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"DateTime","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"result_time","display":"{round_session}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"  ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID: ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_id","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_desc","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We are currently unable to retrieve the logs from Kibana on our end.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Your assistance in providing these logs at the earliest would be greatly appreciated.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thank you for your support.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Best Regards,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Technical Support Engineer.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Dear Team,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Request:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Please provide the BET/BET_RESULT/END_RESULT/REFUND logs for the following details.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_id","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"DateTime","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":": ","type":"text","version":1},{"type":"field","version":1,"keyName":"result_time","display":"{round_date_time}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"  ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID: ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_id","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_name","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"We are currently unable to retrieve the logs from Kibana on our end.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Your assistance in providing these logs at the earliest would be greatly appreciated.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Thank you for your support.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Best Regards,","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"LC Technical Support Engineer.","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
       </c>
       <c r="G7" t="str">
         <v>true</v>
@@ -677,7 +677,7 @@
         <v>2026-04-07T03:40:50.147Z</v>
       </c>
       <c r="J7" t="str">
-        <v>2026-05-12T05:01:32.467Z</v>
+        <v>2026-05-12T12:07:31.991Z</v>
       </c>
     </row>
   </sheetData>
@@ -742,7 +742,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>casino_desc</v>
+        <v>casino_name</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
       </c>
       <c r="E3" t="str">
         <v>{casino_name}</v>
@@ -751,7 +757,7 @@
         <v>2026-04-04T16:58:32.759Z</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-08T20:33:22.068Z</v>
+        <v>2026-05-12T12:07:09.921Z</v>
       </c>
     </row>
     <row r="4">
@@ -922,13 +928,13 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>{round_session}</v>
+        <v>{round_date_time}</v>
       </c>
       <c r="F12" t="str">
         <v>2026-04-07T03:43:36.650Z</v>
       </c>
       <c r="G12" t="str">
-        <v>2026-05-12T05:00:51.180Z</v>
+        <v>2026-05-12T12:04:11.491Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update resolution template file
</commit_message>
<xml_diff>
--- a/db_storage/resolution_template.xlsx
+++ b/db_storage/resolution_template.xlsx
@@ -529,19 +529,25 @@
         <v>All</v>
       </c>
       <c r="D2" t="str">
-        <v>Resolution Summary</v>
+        <v>SAP</v>
       </c>
       <c r="E2" t="str">
         <v>General Round Check</v>
       </c>
       <c r="F2" t="str">
-        <v>{"root":{"children":[{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Issue:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Steps to Reproduce:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_id","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_name","display":"{casino_name}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_id","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Player ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"user_id","display":"{user_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"game_id","display":"{game_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Live","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Internal Investigation:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Upon investigation, we have found that:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"BET Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"bet_details","display":"{bet_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Transaction Details:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"transaction_details","display":"{transaction_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Next Action:","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Communicating with the operator","type":"text","version":1},{"detail":0,"format":16,"mode":"normal","style":"","text":".","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+        <v>{"root":{"children":[{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Issue:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Steps to Reproduce:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_id","display":"{casino_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Casino Name:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"casino_name","display":"{casino_name}"},{"detail":0,"format":1,"mode":"normal","style":"","text":" ","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Operator: ","type":"text","version":1},{"type":"field","version":1,"keyName":"Wallet_Type","display":"{wallet_type}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Round ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"round_id","display":"{round_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Player ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"user_id","display":"{user_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Game ID:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" ","type":"text","version":1},{"type":"field","version":1,"keyName":"game_id","display":"{game_id}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Env:","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":" Live","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Internal Investigation:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""},{"children":[{"detail":0,"format":0,"mode":"normal","style":"","text":"Upon investigation, we have found that:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"BET Details","type":"text","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":":","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"bet_details","display":"{bet_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":1,"mode":"normal","style":"","text":"Transaction Details:","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":1,"textStyle":""},{"children":[{"type":"field","version":1,"keyName":"transaction_details","display":"{transaction_details}"}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":0,"textStyle":""},{"children":[{"detail":0,"format":9,"mode":"normal","style":"","text":"Next Action:","type":"text","version":1},{"type":"linebreak","version":1},{"detail":0,"format":0,"mode":"normal","style":"","text":"Communicating with the operator","type":"text","version":1},{"detail":0,"format":16,"mode":"normal","style":"","text":".","type":"text","version":1}],"direction":null,"format":"","indent":0,"type":"paragraph","version":1,"textFormat":9,"textStyle":""}],"direction":null,"format":"","indent":0,"type":"root","version":1}}</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
       </c>
       <c r="I2" t="str">
         <v>2026-04-04T15:50:25.541Z</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-05-12T12:15:18.799Z</v>
+        <v>2026-05-15T13:56:51.436Z</v>
       </c>
     </row>
     <row r="3">
@@ -689,7 +695,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -725,7 +731,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>https://supporttools.pragmaticplaylive.net/portal/casino-details/{casino_id}</v>
       </c>
       <c r="E2" t="str">
         <v>{casino_id}</v>
@@ -734,7 +740,7 @@
         <v>2026-04-04T16:55:20.125Z</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-13T14:57:01.585Z</v>
+        <v>2026-05-15T13:52:20.586Z</v>
       </c>
     </row>
     <row r="3">
@@ -771,7 +777,7 @@
         <v>1</v>
       </c>
       <c r="D4" t="str">
-        <v>http://localhost:3000/round-activity?roundId={round_id}</v>
+        <v>https://supporttools.pragmaticplaylive.net/portal/round-activity?roundId={round_id}</v>
       </c>
       <c r="E4" t="str">
         <v>{round_id}</v>
@@ -780,7 +786,7 @@
         <v>2026-04-04T16:58:49.682Z</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-04-13T14:57:49.396Z</v>
+        <v>2026-05-15T13:51:29.000Z</v>
       </c>
     </row>
     <row r="5">
@@ -811,7 +817,7 @@
         <v>1</v>
       </c>
       <c r="D6" t="str">
-        <v>http://localhost:3000/round-activity?gameId={game_id}&amp;userId={user_id}</v>
+        <v>https://supporttools.pragmaticplaylive.net/portal/round-activity?gameId={game_id}&amp;userId={user_id}</v>
       </c>
       <c r="E6" t="str">
         <v>{game_id}</v>
@@ -820,7 +826,7 @@
         <v>2026-04-04T16:59:51.282Z</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-04-13T16:10:15.279Z</v>
+        <v>2026-05-15T13:51:41.403Z</v>
       </c>
     </row>
     <row r="7">
@@ -937,9 +943,32 @@
         <v>2026-05-12T12:04:11.491Z</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Wallet_Type</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v>{wallet_type}</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2026-05-15T13:54:18.811Z</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2026-05-15T13:54:18.811Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1177,13 +1206,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Resolution Summary</v>
+        <v>SAP</v>
       </c>
       <c r="C2" t="str">
         <v>2026-04-06T13:16:07.715Z</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-04-06T13:16:07.715Z</v>
+        <v>2026-05-15T12:12:31.210Z</v>
       </c>
     </row>
     <row r="3">
@@ -1243,7 +1272,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>

</xml_diff>